<commit_message>
Verificacion de avances: reporte para WFP/MIMI + tabla FC despensa completa (98 celdas)
- docs/20260827 Reporte_avances_ENGIH_Secciones_2_y_3A.md: los 2 avances del correo con numeros verificados + estado de la tarea de unidades (79.4% cubierto, 98 celdas pendientes, preguntas D1/D2).
- crosswalk_variedad_SEC2.xlsx: FC_pendientes reescrita con las 98 celdas alimento×unidad completas (9,629 registros; 61 con referencia propuesta); correcciones de notas (codigo 31 = 23 registros; catalogo = 0.06%).
- PLAN + README: '~20 celdas' -> 98 celdas (28 principales cubren ~96%); codigos sin nombre = 35 registros; 199 registros Sec 2 sin unidad (0.4%).

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/raw/crosswalk_variedad_SEC2.xlsx
+++ b/data/raw/crosswalk_variedad_SEC2.xlsx
@@ -448,9 +448,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -493,9 +491,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -506,13 +502,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   catálogo (0.09%) + 5 códigos sin descripción (0.07%) = 46 filas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+          <t xml:space="preserve">   catálogo (0.06%) + 5 códigos sin descripción (0.07%) = 46 filas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -583,9 +577,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -607,9 +599,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -627,13 +617,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   de pesos de porciones). Con 30 alimentos la tabla completa es ~20 celdas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
+          <t xml:space="preserve">   de pesos de porciones). Con 30 alimentos la tabla completa es 98 celdas (9,629 registros; las 28 principales cubren ~96% de esos registros).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -776,8 +764,6 @@
           <t>Unidad 2, Libra 2, Onza 1</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -896,7 +882,6 @@
       <c r="N4" t="b">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -947,7 +932,6 @@
       <c r="N5" t="b">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1053,7 +1037,6 @@
       <c r="N7" t="b">
         <v>0</v>
       </c>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1214,7 +1197,6 @@
       <c r="N10" t="b">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1320,7 +1302,6 @@
       <c r="N12" t="b">
         <v>0</v>
       </c>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1536,7 +1517,6 @@
       <c r="N16" t="b">
         <v>0</v>
       </c>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1697,7 +1677,6 @@
       <c r="N19" t="b">
         <v>0</v>
       </c>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1774,8 +1753,6 @@
           <t>Gramos 209, Onza 98, Lata 23</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -1839,7 +1816,6 @@
       <c r="N22" t="b">
         <v>0</v>
       </c>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1861,8 +1837,6 @@
           <t>Onza 227, Gramos 203, Lata 32</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -1926,7 +1900,6 @@
       <c r="N24" t="b">
         <v>0</v>
       </c>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1977,7 +1950,6 @@
       <c r="N25" t="b">
         <v>0</v>
       </c>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2028,7 +2000,6 @@
       <c r="N26" t="b">
         <v>0</v>
       </c>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2079,7 +2050,6 @@
       <c r="N27" t="b">
         <v>0</v>
       </c>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2211,8 +2181,6 @@
           <t>Onza 384, Gramos 204, Libra 111</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2357,8 +2325,6 @@
           <t>Libra 7, Gramos 6, Unidad 5</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2369,7 +2335,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Sin descripcion en encuesta ni catalogo (10 registros). Verificar contra BCRD.</t>
+          <t>Sin descripcion en encuesta ni catalogo (23 registros). Verificar contra BCRD.</t>
         </is>
       </c>
     </row>
@@ -2396,8 +2362,6 @@
       <c r="F34" t="n">
         <v>32</v>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2432,8 +2396,6 @@
           <t>Libra 2, Gramos 1, Unidad 1</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2471,8 +2433,6 @@
       <c r="F36" t="n">
         <v>34</v>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2510,8 +2470,6 @@
       <c r="F37" t="n">
         <v>35</v>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2546,8 +2504,6 @@
           <t>Unidad 1</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2640,8 +2596,6 @@
           <t>Onza 1</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -2766,7 +2720,6 @@
       <c r="N42" t="b">
         <v>0</v>
       </c>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2878,7 +2831,6 @@
       <c r="N44" t="b">
         <v>0</v>
       </c>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2903,8 +2855,6 @@
       <c r="F45" t="n">
         <v>73</v>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>requiere_revision</t>
@@ -3046,44 +2996,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>id_variedad</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>id_unidad_medida</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>n_registros</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>referencia_sugerida_g</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>nota</t>
         </is>
@@ -3092,18 +3048,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TODOS los valores son PLACEHOLDERS a validar antes de usar (BCRD/MIMI o tabla de pesos de porciones).</t>
+          <t>HUEVOS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2725</v>
+      </c>
+      <c r="F2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>con cáscara; el PC (EDIBLE INCAP) descuenta la cáscara</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HUEVOS</t>
+          <t>PLÁTANO VERDE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3111,25 +3089,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2725</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>con cascara; el PC (EDIBLE INCAP) descuenta la cascara</t>
+        <v>1729</v>
+      </c>
+      <c r="F3" t="n">
+        <v>300</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>con cáscara</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PANES</t>
+          <t>GUINEITO VERDE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3137,25 +3118,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1188</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>pan de agua</t>
+        <v>1355</v>
+      </c>
+      <c r="F4" t="n">
+        <v>80</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>con cáscara</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GALLETAS SALADAS</t>
+          <t>PANES</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3163,21 +3147,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>605</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>1188</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>pan de agua</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GALLETAS DULCES</t>
+          <t>GALLETAS SALADAS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3185,21 +3176,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>374</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
+        <v>605</v>
+      </c>
+      <c r="F6" t="n">
         <v>12</v>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>galleta estándar</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PLÁTANO VERDE</t>
+          <t>GALLETAS DULCES</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3207,66 +3205,75 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1729</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>300</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>con cascara</t>
+        <v>374</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>galleta estándar</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLÁTANO VERDE</t>
+          <t>CHOCOLATE O COCOA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Racimo</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>6 unidades aprox.</t>
+        <v>187</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>barra</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PLÁTANO VERDE</t>
+          <t>HABICHUELAS SUELTAS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mano</t>
+          <t>Jarro</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E9" t="n">
-        <v>600</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>5-6 unidades aprox.</t>
+        <v>83</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>jarro ~1.5 L; validar</t>
         </is>
       </c>
     </row>
@@ -3281,18 +3288,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Mano</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1355</v>
+        <v>66</v>
       </c>
       <c r="E10" t="n">
         <v>80</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>con cascara</t>
+      <c r="F10" t="n">
+        <v>480</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6 unidades aprox.</t>
         </is>
       </c>
     </row>
@@ -3307,330 +3317,2464 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mano</t>
+          <t>Racimo</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E11" t="n">
-        <v>480</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>6 unidades aprox.</t>
+        <v>78</v>
+      </c>
+      <c r="F11" t="n">
+        <v>960</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>12 unidades aprox.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GUINEITO VERDE</t>
+          <t>CHOCOLATE O COCOA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Racimo</t>
+          <t>Tableta</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="E12" t="n">
-        <v>960</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>12 unidades aprox.</t>
+        <v>76</v>
+      </c>
+      <c r="F12" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>tableta</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ATUN / SARDINAS / PICA PICA (latas)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>20,21,22,23</t>
-        </is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>16</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lata</t>
+          <t>Botella</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>205</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
-        <v>160</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>lata estandar; validar peso neto tipico RD</t>
+        <v>72</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>botella 1 L; validar</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LECHE EN POLVO</t>
+          <t>LECHE LÍQUIDA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lata</t>
+          <t>Botella</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="E14" t="n">
-        <v>400</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>lata estandar</t>
+        <v>65</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>validar</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHOCOLATE O COCOA</t>
+          <t>ATÚN EN ACEITE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Lata</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>187</v>
+        <v>63</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>barra</t>
+        <v>60</v>
+      </c>
+      <c r="F15" t="n">
+        <v>160</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>lata estándar; validar peso neto típico RD</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SALAMI</t>
+          <t>PLÁTANO VERDE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Unidad / Pieza</t>
+          <t>Racimo</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="E16" t="n">
-        <v>25</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>rebanada</t>
+        <v>58</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>6 unidades aprox.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>PLÁTANO VERDE</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Mano</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="E17" t="n">
-        <v>500</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>pieza; validar (impacto alto)</t>
+        <v>48</v>
+      </c>
+      <c r="F17" t="n">
+        <v>600</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-6 unidades aprox.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PESCADO</t>
+          <t>ATÚN EN AGUA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Lata</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="E18" t="n">
-        <v>200</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>filete/pieza</t>
+        <v>44</v>
+      </c>
+      <c r="F18" t="n">
+        <v>160</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PAPAS</t>
+          <t>ARROZ</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Jarro</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>150</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>papa mediana</t>
+        <v>43</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>jarro ~1.5 L; validar</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ARROZ</t>
+          <t>PAPAS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Jarro</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>jarro ~1.5 L; validar</t>
+        <v>40</v>
+      </c>
+      <c r="F20" t="n">
+        <v>150</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>papa mediana</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HABICHUELAS SUELTAS</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Jarro</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>jarro ~1.5 L; validar</t>
+        <v>39</v>
+      </c>
+      <c r="F21" t="n">
+        <v>500</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>pieza; validar (impacto alto)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CARNE DE RES</t>
+          <t>HARÍNA DE MAÍZ</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Paquete</t>
+          <t>Funda</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="E22" t="n">
+        <v>38</v>
+      </c>
+      <c r="F22" t="n">
         <v>500</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>paquete supermercado</t>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>funda de masa; validar</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>16</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pote</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>87</v>
+      </c>
+      <c r="E23" t="n">
+        <v>36</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GALLETAS SALADAS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" t="n">
+        <v>35</v>
+      </c>
+      <c r="F24" t="n">
+        <v>120</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>paquete ~10 galletas; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>FIEDOS O SPAGUETTIS (PASTAS)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>56</v>
+      </c>
+      <c r="E25" t="n">
+        <v>33</v>
+      </c>
+      <c r="F25" t="n">
+        <v>500</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>funda estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PICA PICA</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>21</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>63</v>
+      </c>
+      <c r="E26" t="n">
+        <v>32</v>
+      </c>
+      <c r="F26" t="n">
+        <v>160</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>32</v>
+      </c>
+      <c r="F27" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>rebanada</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LECHE EN POLVO</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>63</v>
+      </c>
+      <c r="E28" t="n">
+        <v>31</v>
+      </c>
+      <c r="F28" t="n">
+        <v>400</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>18</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>81</v>
+      </c>
+      <c r="E29" t="n">
+        <v>29</v>
+      </c>
+      <c r="F29" t="n">
+        <v>25</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>pieza/rebanada</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LECHE EN POLVO</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>14</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>56</v>
+      </c>
+      <c r="E30" t="n">
+        <v>24</v>
+      </c>
+      <c r="F30" t="n">
+        <v>400</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>funda/brick; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MANTEQUILLA</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>17</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tarro</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>105</v>
+      </c>
+      <c r="E31" t="n">
+        <v>24</v>
+      </c>
+      <c r="F31" t="n">
+        <v>200</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FIEDOS O SPAGUETTIS (PASTAS)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" t="n">
+        <v>24</v>
+      </c>
+      <c r="F32" t="n">
+        <v>500</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SARDINAS EN AGUA</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>19</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>63</v>
+      </c>
+      <c r="E33" t="n">
+        <v>23</v>
+      </c>
+      <c r="F33" t="n">
+        <v>160</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FIEDOS O SPAGUETTIS (PASTAS)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>22</v>
+      </c>
+      <c r="F34" t="n">
+        <v>100</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PANES</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Rebanada</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>93</v>
+      </c>
+      <c r="E35" t="n">
+        <v>22</v>
+      </c>
+      <c r="F35" t="n">
+        <v>50</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>rebanada estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>56</v>
+      </c>
+      <c r="E36" t="n">
+        <v>21</v>
+      </c>
+      <c r="F36" t="n">
+        <v>500</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>funda estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>30</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pote</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>87</v>
+      </c>
+      <c r="E37" t="n">
+        <v>19</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>18</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Pedazo</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>79</v>
+      </c>
+      <c r="E38" t="n">
+        <v>17</v>
+      </c>
+      <c r="F38" t="n">
+        <v>50</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PANES</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Rodaja</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>94</v>
+      </c>
+      <c r="E39" t="n">
+        <v>17</v>
+      </c>
+      <c r="F39" t="n">
+        <v>50</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>rodaja estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SARDINAS EN ACEITE</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>63</v>
+      </c>
+      <c r="E40" t="n">
+        <v>16</v>
+      </c>
+      <c r="F40" t="n">
+        <v>160</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SARDINAS EN AGUA</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>19</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PESCADO</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>11</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>11</v>
+      </c>
+      <c r="F42" t="n">
+        <v>200</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>filete/pieza; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>30</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sobre</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>98</v>
+      </c>
+      <c r="E43" t="n">
+        <v>11</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>por definir (sobre individual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>16</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Tercia</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>107</v>
+      </c>
+      <c r="E44" t="n">
+        <v>11</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>medida tradicional; por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>16</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>56</v>
+      </c>
+      <c r="E45" t="n">
+        <v>10</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GALLETAS DULCES</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" t="n">
+        <v>10</v>
+      </c>
+      <c r="F46" t="n">
+        <v>120</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>paquete ~10 galletas; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SARDINAS EN ACEITE</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>20</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="n">
+        <v>9</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CARNE DE RES</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>8</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8</v>
+      </c>
+      <c r="F48" t="n">
+        <v>500</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>paquete supermercado; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>30</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>17</v>
+      </c>
+      <c r="E49" t="n">
+        <v>7</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LECHE EN POLVO</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>14</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sobre</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>98</v>
+      </c>
+      <c r="E50" t="n">
+        <v>6</v>
+      </c>
+      <c r="F50" t="n">
+        <v>25</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>sachet; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>30</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tarro</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>105</v>
+      </c>
+      <c r="E51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PANES</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Viga</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>117</v>
+      </c>
+      <c r="E52" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>viga (pan grande); por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PANES</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Pedazo</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>79</v>
+      </c>
+      <c r="E53" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>MANTEQUILLA</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>17</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Barrita</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>14</v>
+      </c>
+      <c r="E54" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" t="n">
+        <v>25</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>barra estándar</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>18</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Cuarto</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>45</v>
+      </c>
+      <c r="E55" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" t="n">
+        <v>125</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>cuarto de pieza; por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MANTEQUILLA</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>17</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Cucharada</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>49</v>
+      </c>
+      <c r="E56" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" t="n">
+        <v>14</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>1 cda ≈ 14 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>18</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Trozo</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>111</v>
+      </c>
+      <c r="E57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" t="n">
+        <v>100</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LECHE EN POLVO</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>14</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>4</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>16</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>3</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SALAMI</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>18</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Pié</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>80</v>
+      </c>
+      <c r="E60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" t="n">
+        <v>25</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>HABICHUELAS SUELTAS</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>27</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>56</v>
+      </c>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>funda ~1 kg; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>30</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>56</v>
+      </c>
+      <c r="E62" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>HABICHUELAS ENLATADAS</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>28</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>63</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="n">
+        <v>400</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>lata estándar; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>GUINEITO VERDE</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>25</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Quintal</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>90</v>
+      </c>
+      <c r="E64" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" t="n">
+        <v>47600</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>1 quintal = 47.6 kg (exacto por definición)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>HARÍNA DE MAÍZ</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>8</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="n">
+        <v>500</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>HARÍNA DE MAÍZ</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" t="n">
+        <v>100</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>GALLETAS SALADAS</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>63</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>por definir (lata de galletas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MANTEQUILLA</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>17</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Pote</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>87</v>
+      </c>
+      <c r="E68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>MARISCOS</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B69" t="n">
         <v>12</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Paquete</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D69" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
         <v>400</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>PESCADO</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>11</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>56</v>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ARROZ</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>7</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Saco</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>97</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>saco 50 lb; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Sobre</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>98</v>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>PESCADO</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>11</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Pedazo</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>79</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>63</v>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Tarro</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>105</v>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>GALLETAS DULCES</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>63</v>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>GALLETAS SALADAS</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>56</v>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>5</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>GALLETAS DULCES</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>56</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>8</v>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>AVENA</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>5</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Pote</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>87</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>16</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sobre</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>98</v>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ACEITE</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>16</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Tarro</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>105</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>MANTEQUILLA</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>17</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>HUEVOS</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>15</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Cartón</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>31</v>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>cartón de 30 huevos (30 × 60 g); validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>LECHE LÍQUIDA</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>13</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>63</v>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>LECHE LÍQUIDA</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>13</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Cartón</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>31</v>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>cartón 1 L; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>LECHE LÍQUIDA</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>13</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Frasco</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>55</v>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>500</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>por validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>PAPAS</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>26</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Pila</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>82</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>PAPAS</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>26</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Mano</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>66</v>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>por definir (~500 g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>PLÁTANO VERDE</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>24</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Saco</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>97</v>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>por definir (saco de carga)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>HABICHUELAS SUELTAS</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>27</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>30</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>8</v>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>HABICHUELAS SUELTAS</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>27</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>63</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" t="n">
+        <v>400</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>lata estándar de frijol; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>AZUCARES</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>29</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Funda</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>56</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>funda ~1 kg; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>30</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Barrita</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>14</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="n">
+        <v>20</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>barrita; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>30</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>23</v>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>30</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>63</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>CHOCOLATE O COCOA</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>30</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Tercia</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>107</v>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>